<commit_message>
[데이터] Stage 데이터에 StagePrefabPath 컬럼 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Stage.xlsx
+++ b/Development/Common/GameData/Stage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB08CE8-B944-4F68-B54A-E274EA40E518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61D86843-D3EE-42A3-BC3D-5ABE93A73AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39840" yWindow="6615" windowWidth="27360" windowHeight="14340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2070" yWindow="2190" windowWidth="31605" windowHeight="17295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stage" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="50">
   <si>
     <t>데이터이름</t>
   </si>
@@ -206,27 +206,16 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Field1</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Field2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Field3</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dungeon1</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dungeon2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dungeon3</t>
+    <t>StagePrefabPath</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stage 프리팹 경로.
+루트경로: Assets/Resources/</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Prefabs/Stages/Town</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -690,7 +679,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.25" style="12" customWidth="1"/>
@@ -699,13 +688,14 @@
     <col min="4" max="4" width="26" style="3" customWidth="1"/>
     <col min="5" max="5" width="23.625" style="3" customWidth="1"/>
     <col min="6" max="6" width="16.25" style="3" customWidth="1"/>
-    <col min="7" max="7" width="46.875" style="3" customWidth="1"/>
-    <col min="8" max="8" width="19.25" style="3" customWidth="1"/>
-    <col min="9" max="9" width="18.75" style="3" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="3"/>
+    <col min="7" max="7" width="28.625" style="3" customWidth="1"/>
+    <col min="8" max="8" width="46.875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="19.25" style="3" customWidth="1"/>
+    <col min="10" max="10" width="18.75" style="3" customWidth="1"/>
+    <col min="11" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -713,7 +703,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -733,13 +723,16 @@
         <v>33</v>
       </c>
       <c r="G2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:8" s="7" customFormat="1" ht="132" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" s="7" customFormat="1" ht="132" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>3</v>
       </c>
@@ -751,13 +744,16 @@
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -777,13 +773,16 @@
         <v>17</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I4" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -802,10 +801,13 @@
         <v>18</v>
       </c>
       <c r="H5" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -818,8 +820,9 @@
       </c>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I6" s="8"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -833,11 +836,12 @@
         <v>20</v>
       </c>
       <c r="G7" s="8"/>
-      <c r="H7" s="8">
+      <c r="H7" s="8"/>
+      <c r="I7" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>10</v>
       </c>
@@ -857,13 +861,16 @@
         <v>32</v>
       </c>
       <c r="G8" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="I8" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>1</v>
       </c>
@@ -879,11 +886,11 @@
       <c r="F9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="3">
+      <c r="I9" s="3">
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>100</v>
       </c>
@@ -894,13 +901,16 @@
         <v>34</v>
       </c>
       <c r="G10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H10" s="3">
+      <c r="I10" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>101</v>
       </c>
@@ -911,13 +921,16 @@
         <v>35</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H11" s="3">
+        <v>49</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <v>102</v>
       </c>
@@ -928,13 +941,16 @@
         <v>35</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H12" s="3">
+        <v>49</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I12" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <v>103</v>
       </c>
@@ -947,11 +963,14 @@
       <c r="G13" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="H13" s="3">
+      <c r="H13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I13" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <v>104</v>
       </c>
@@ -962,13 +981,16 @@
         <v>36</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="H14" s="3">
+        <v>49</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I14" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <v>105</v>
       </c>
@@ -979,13 +1001,16 @@
         <v>36</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="H15" s="3">
+        <v>49</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I15" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <v>106</v>
       </c>
@@ -996,9 +1021,12 @@
         <v>36</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H16" s="3">
+        <v>49</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I16" s="3">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[데이터] Stage 데이터에 ScriptName 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Stage.xlsx
+++ b/Development/Common/GameData/Stage.xlsx
@@ -1,222 +1,213 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3981E42-A509-4AC9-8226-8ECC734C0C87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D07A51C5-DBF7-49F4-AEC1-0F809E7787F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2415" yWindow="2535" windowWidth="31605" windowHeight="17295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stage" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="61">
   <si>
     <t>데이터이름</t>
   </si>
   <si>
+    <t>Stage</t>
+  </si>
+  <si>
     <t>컬럼설명</t>
   </si>
   <si>
     <t>키값</t>
   </si>
   <si>
+    <t>메모</t>
+  </si>
+  <si>
+    <t>스테이지이름</t>
+  </si>
+  <si>
+    <t>참고</t>
+  </si>
+  <si>
+    <t>스테이지타입</t>
+  </si>
+  <si>
+    <t>NavMesh</t>
+  </si>
+  <si>
+    <t>섹터 크기</t>
+  </si>
+  <si>
+    <t>스크립트1</t>
+  </si>
+  <si>
+    <t>스크립트2</t>
+  </si>
+  <si>
+    <t>스크립트3</t>
+  </si>
+  <si>
     <t>컬럼설명세부</t>
   </si>
   <si>
-    <t>Target</t>
-  </si>
-  <si>
-    <t>all</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>DataType</t>
-  </si>
-  <si>
-    <t>DefaultValue</t>
-  </si>
-  <si>
-    <t>컬럼명</t>
-  </si>
-  <si>
-    <t>Key</t>
-  </si>
-  <si>
-    <t>DataTypeDetail</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>메모</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>참고</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Name</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>client</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>all</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>string</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>enum</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>None</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>참고이름</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Stage</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>마을</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>스테이지이름</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>스테이지 특징 기입</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>필드1</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>필드2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>필드3</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>던전1</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>던전2</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>던전3</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>StageType</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>스테이지타입</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Town</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Field</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Dungeon</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>섹터 크기</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>섹터 크기는 한 변이 sectorSize인 정사각형임</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>캐릭터 선택창</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>게임서버당 1개씩 존재, 게임서버 시작할때 생성됨</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>System</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>sectorSize</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>NavMesh</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>NavMeshFileName</t>
-    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stage 프리팹 경로.
+루트경로: Assets/Resources/</t>
   </si>
   <si>
     <t>NavMesh 파일 이름.
 - 서버의 NavMesh 파일 경로: Server/OUTPUT/Map/NavMesh/파일명.bin
 - 클라의 NavMesh 파일 경로: Client/Assets/StreamingAssets/NavMesh/파일명.bin
 - 서버의 NavMesh meta정보 파일(월드크기 등 정보가 있음) 경로: Server/OUTPUT/Map/NavMesh/파일명.navmeta.json</t>
+  </si>
+  <si>
+    <t>섹터 크기는 한 변이 sectorSize인 정사각형임</t>
+  </si>
+  <si>
+    <t>이 Stage 에서 로드할 Lua 스크립트(Map/StageScript/&lt;이름&gt;.lua). 비우면 없음.</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>all</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>client</t>
+  </si>
+  <si>
+    <t>server</t>
+  </si>
+  <si>
+    <t>DataType</t>
+  </si>
+  <si>
+    <t>int32</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>enum</t>
+  </si>
+  <si>
+    <t>float</t>
+  </si>
+  <si>
+    <t>DataTypeDetail</t>
+  </si>
+  <si>
+    <t>StageType</t>
+  </si>
+  <si>
+    <t>DefaultValue</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>컬럼명</t>
+  </si>
+  <si>
+    <t>Key</t>
+  </si>
+  <si>
+    <t>참고이름</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>StagePrefabPath</t>
+  </si>
+  <si>
+    <t>NavMeshFileName</t>
+  </si>
+  <si>
+    <t>sectorSize</t>
+  </si>
+  <si>
+    <t>ScriptName1</t>
+  </si>
+  <si>
+    <t>ScriptName2</t>
+  </si>
+  <si>
+    <t>ScriptName3</t>
+  </si>
+  <si>
+    <t>캐릭터 선택창</t>
+  </si>
+  <si>
+    <t>게임서버당 1개씩 존재, 게임서버 시작할때 생성됨</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>마을</t>
+  </si>
+  <si>
+    <t>Town</t>
+  </si>
+  <si>
+    <t>Prefabs/Stages/Town</t>
+  </si>
+  <si>
+    <t>town</t>
+  </si>
+  <si>
+    <t>town_event</t>
+  </si>
+  <si>
+    <t>필드1</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>필드2</t>
+  </si>
+  <si>
+    <t>필드3</t>
+  </si>
+  <si>
+    <t>던전1</t>
+  </si>
+  <si>
+    <t>Dungeon</t>
+  </si>
+  <si>
+    <t>던전2</t>
+  </si>
+  <si>
+    <t>던전3</t>
+  </si>
+  <si>
+    <t>추가 스크립트(이벤트 등). 기본 스크립트 수정 없이 로직 추가.</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>StagePrefabPath</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Stage 프리팹 경로.
-루트경로: Assets/Resources/</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>Prefabs/Stages/Town</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>int32</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>float</t>
+    <t>추가 스크립트2</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -353,10 +344,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -680,7 +671,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.25" style="12" customWidth="1"/>
@@ -692,140 +683,181 @@
     <col min="7" max="7" width="28.625" style="3" customWidth="1"/>
     <col min="8" max="8" width="46.875" style="3" customWidth="1"/>
     <col min="9" max="9" width="19.25" style="3" customWidth="1"/>
-    <col min="10" max="10" width="18.75" style="3" customWidth="1"/>
-    <col min="11" max="16384" width="9" style="3"/>
+    <col min="10" max="10" width="26.375" style="3" customWidth="1"/>
+    <col min="11" max="11" width="27.125" style="3" customWidth="1"/>
+    <col min="12" max="12" width="26.75" style="3" customWidth="1"/>
+    <col min="13" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="H2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:12" s="7" customFormat="1" ht="132" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
         <v>13</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" s="7" customFormat="1" ht="132" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>3</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
       <c r="E3" s="6" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I4" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="L4" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="E5" s="8"/>
       <c r="F5" s="8" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G6" s="8"/>
       <c r="H6" s="8"/>
       <c r="I6" s="8"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B7" s="8">
         <v>0</v>
@@ -834,198 +866,216 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
       <c r="I7" s="8">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+    </row>
+    <row r="8" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="I8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="K8" s="10" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="L8" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>1</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I9" s="3">
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>100</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="G10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I10" s="3">
         <v>10</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>101</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="G11" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I11" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <v>102</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="G12" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I12" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <v>103</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="G13" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H13" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I13" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <v>104</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="G14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I14" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <v>105</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="G15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I15" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <v>106</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>30</v>
+        <v>58</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>35</v>
+        <v>56</v>
       </c>
       <c r="G16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="I16" s="3">
         <v>10</v>
@@ -1034,6 +1084,6 @@
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[데이터] Stage 데이터에 StageLayoutFileName 컬럼 추가
</commit_message>
<xml_diff>
--- a/Development/Common/GameData/Stage.xlsx
+++ b/Development/Common/GameData/Stage.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\project\MMOGameServerProject\Development\Common\GameData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\project\MMOGameServerProject\Development\Common\GameData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D07A51C5-DBF7-49F4-AEC1-0F809E7787F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0260CF-0BF6-4281-B3E9-DDF879579CB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="63">
   <si>
     <t>데이터이름</t>
   </si>
@@ -176,9 +176,6 @@
     <t>town</t>
   </si>
   <si>
-    <t>town_event</t>
-  </si>
-  <si>
     <t>필드1</t>
   </si>
   <si>
@@ -208,6 +205,18 @@
   </si>
   <si>
     <t>추가 스크립트2</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Stage 상의 Spawner, EventArea 위치를 담고 있는 StageLayout 파일 이름.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StageLayout</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>StageLayoutFileName</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -671,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.25" style="12" customWidth="1"/>
@@ -681,15 +690,16 @@
     <col min="5" max="5" width="23.625" style="3" customWidth="1"/>
     <col min="6" max="6" width="16.25" style="3" customWidth="1"/>
     <col min="7" max="7" width="28.625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="46.875" style="3" customWidth="1"/>
-    <col min="9" max="9" width="19.25" style="3" customWidth="1"/>
-    <col min="10" max="10" width="26.375" style="3" customWidth="1"/>
-    <col min="11" max="11" width="27.125" style="3" customWidth="1"/>
-    <col min="12" max="12" width="26.75" style="3" customWidth="1"/>
-    <col min="13" max="16384" width="9" style="3"/>
+    <col min="8" max="8" width="44.5" style="3" customWidth="1"/>
+    <col min="9" max="9" width="21.75" style="3" customWidth="1"/>
+    <col min="10" max="10" width="19.25" style="3" customWidth="1"/>
+    <col min="11" max="11" width="26.375" style="3" customWidth="1"/>
+    <col min="12" max="12" width="27.125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="26.75" style="3" customWidth="1"/>
+    <col min="14" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -697,7 +707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -723,19 +733,22 @@
         <v>8</v>
       </c>
       <c r="I2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="L2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="M2" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="7" customFormat="1" ht="132" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" s="7" customFormat="1" ht="132" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>13</v>
       </c>
@@ -753,19 +766,22 @@
         <v>16</v>
       </c>
       <c r="I3" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="K3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="L3" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="M3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="L3" s="6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -794,7 +810,7 @@
         <v>20</v>
       </c>
       <c r="J4" s="8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="K4" s="8" t="s">
         <v>23</v>
@@ -802,8 +818,11 @@
       <c r="L4" s="8" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M4" s="8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>24</v>
       </c>
@@ -825,10 +844,10 @@
         <v>26</v>
       </c>
       <c r="I5" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="J5" s="8" t="s">
         <v>28</v>
-      </c>
-      <c r="J5" s="8" t="s">
-        <v>26</v>
       </c>
       <c r="K5" s="8" t="s">
         <v>26</v>
@@ -836,8 +855,11 @@
       <c r="L5" s="8" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M5" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>29</v>
       </c>
@@ -854,8 +876,9 @@
       <c r="J6" s="8"/>
       <c r="K6" s="8"/>
       <c r="L6" s="8"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="M6" s="8"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>31</v>
       </c>
@@ -870,14 +893,15 @@
       </c>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
-      <c r="I7" s="8">
+      <c r="I7" s="8"/>
+      <c r="J7" s="8">
         <v>0</v>
       </c>
-      <c r="J7" s="8"/>
       <c r="K7" s="8"/>
       <c r="L7" s="8"/>
-    </row>
-    <row r="8" spans="1:12" s="11" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="M7" s="8"/>
+    </row>
+    <row r="8" spans="1:13" s="11" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>33</v>
       </c>
@@ -903,19 +927,22 @@
         <v>38</v>
       </c>
       <c r="I8" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="J8" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="K8" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="K8" s="10" t="s">
+      <c r="L8" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="M8" s="10" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>1</v>
       </c>
@@ -931,11 +958,11 @@
       <c r="F9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I9" s="3">
+      <c r="J9" s="3">
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>100</v>
       </c>
@@ -951,25 +978,25 @@
       <c r="H10" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I10" s="3">
+      <c r="I10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J10" s="3">
         <v>10</v>
       </c>
-      <c r="J10" s="3" t="s">
+      <c r="K10" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>101</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>48</v>
@@ -977,19 +1004,22 @@
       <c r="H11" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J11" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B12" s="3">
         <v>102</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>48</v>
@@ -997,19 +1027,22 @@
       <c r="H12" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I12" s="3">
+      <c r="I12" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J12" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B13" s="3">
         <v>103</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>48</v>
@@ -1017,19 +1050,22 @@
       <c r="H13" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I13" s="3">
+      <c r="I13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J13" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B14" s="3">
         <v>104</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>56</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>48</v>
@@ -1037,19 +1073,22 @@
       <c r="H14" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I14" s="3">
+      <c r="I14" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J14" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B15" s="3">
         <v>105</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>48</v>
@@ -1057,19 +1096,22 @@
       <c r="H15" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I15" s="3">
+      <c r="I15" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J15" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B16" s="3">
         <v>106</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>48</v>
@@ -1077,7 +1119,10 @@
       <c r="H16" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="3">
+      <c r="I16" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J16" s="3">
         <v>10</v>
       </c>
     </row>

</xml_diff>